<commit_message>
chore: BBS取得 2026-08-11 10:37
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="posts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,7 +482,6 @@
           <t>来ましたー！</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -513,7 +512,6 @@
           <t>気になって来てみました♪</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -546,7 +544,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -579,7 +576,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -610,7 +606,6 @@
           <t>来ましたー</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -643,7 +638,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -674,7 +668,6 @@
           <t>きたよん</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -705,7 +698,6 @@
           <t>きたぞ</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -738,7 +730,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -771,7 +762,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -802,7 +792,6 @@
           <t>はじめてです！</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -833,7 +822,6 @@
           <t>あそびきてみました！</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -864,7 +852,6 @@
           <t>べろべろんちょ</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -897,7 +884,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -930,7 +916,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -963,7 +948,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1064,6 +1048,1286 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>26656</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>22:30:42</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>はなまる</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>久しぶりの</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>日曜日</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>26657</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>22:31:02</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>26658</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>22:33:32</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>大塚</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>きたよー</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>26659</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>22:35:17</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>26660</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>22:46:52</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ゆうと</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>これから行こうと思います</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>26661</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>23:05:54</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>26662</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>23:11:17</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>カー</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>来ました</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26663</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23:11:36</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26664</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>23:45:37</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ミコト、まいまい、テクノ</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ちいかわ</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>トークに</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>26665</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>23:45:57</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>26666</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>00:14:17</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>りょうちゃん</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>バンビ</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>はしご</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>26667</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>00:14:41</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>26668</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>01:18:22</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>らうら</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>少し</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>きたんご</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>26669</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>01:18:40</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>26672</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>19:02:51</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>タツヤ</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>牛タン青味噌</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>持ってきた！！</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>26673</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>19:04:33</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>26674</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>20:00:29</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ふくてゃ、T山</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>激辛祭り！</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>サルサとグリーンカレーあります</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>26675</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>20:00:51</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>イベたのしみに</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>きたよー♪</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>26676</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>20:02:02</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>26677</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>20:02:14</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>26678</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>20:10:13</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Bee</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>今週も</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>楽しみに♪</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>26679</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>20:20:35</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>−、N</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>辛いの苦手だけど</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>頑張ります！</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>26680</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>20:32:57</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>テクノ</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>麻婆豆腐</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>持ってきたー</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>26681</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>20:33:16</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>26682</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>20:33:28</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>26683</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>20:33:41</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>26684</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>20:55:12</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>KUMA</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>大宮バンビから</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>宇都宮は初です！</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>26685</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>20:58:09</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>26686</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>21:17:05</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>コテッチャン</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>来たぜ</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>月曜！！</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>26687</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>21:17:33</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>26688</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>21:40:04</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>なお</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>お土産</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>あるよ♪</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>26689</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>21:46:29</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>26690</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>22:30:38</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ボンタ</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>きてみました</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>26691</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>22:31:02</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>26692</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>22:39:46</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ゆん</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>久々</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>きたよーん</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>26693</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>22:50:20</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>26694</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>22:55:44</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>でで</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>イベ楽しみに</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>きたよー</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>26695</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>22:56:32</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>26696</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>23:23:33</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>いっちゃん</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>きましたー</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>26697</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>23:23:50</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: BBS取得 2026-08-11 23:01 UTC
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1077,7 +1077,6 @@
           <t>日曜日</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1110,7 +1109,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1141,7 +1139,6 @@
           <t>きたよー</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1174,7 +1171,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1205,7 +1201,6 @@
           <t>これから行こうと思います</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1238,7 +1233,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1269,7 +1263,6 @@
           <t>来ました</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1302,7 +1295,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1333,7 +1325,6 @@
           <t>トークに</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1366,7 +1357,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1397,7 +1387,6 @@
           <t>はしご</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1430,7 +1419,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1461,7 +1449,6 @@
           <t>きたんご</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1494,7 +1481,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1525,7 +1511,6 @@
           <t>持ってきた！！</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1558,7 +1543,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1589,7 +1573,6 @@
           <t>サルサとグリーンカレーあります</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1620,7 +1603,6 @@
           <t>きたよー♪</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1653,7 +1635,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1686,7 +1667,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1717,7 +1697,6 @@
           <t>楽しみに♪</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1748,7 +1727,6 @@
           <t>頑張ります！</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1779,7 +1757,6 @@
           <t>持ってきたー</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1812,7 +1789,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1845,7 +1821,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1878,7 +1853,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1909,7 +1883,6 @@
           <t>宇都宮は初です！</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1942,7 +1915,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1973,7 +1945,6 @@
           <t>月曜！！</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2006,7 +1977,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2037,7 +2007,6 @@
           <t>あるよ♪</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2070,7 +2039,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2101,7 +2069,6 @@
           <t>きてみました</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2134,7 +2101,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2165,7 +2131,6 @@
           <t>きたよーん</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2198,7 +2163,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2229,7 +2193,6 @@
           <t>きたよー</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2262,7 +2225,6 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2293,7 +2255,6 @@
           <t>きましたー</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2326,7 +2287,813 @@
 スタッフ一同心よりお待ちしておりますね</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>26716</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>だいち</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>初来店</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>よろしくお願いします
+本日、伺います</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>26717</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>19:02:02</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+風も強いのでお気をつけておこしくださいませ！
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>26718</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>19:51:43</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>ダイチ</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>はじめて</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>きてます！！</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>26720</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>19:56:45</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>26721</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>21:09:24</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>nuri</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>はじめていきます</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>緊張しますが行ってみようと思います！</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>26722</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>21:23:41</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+初めての方でもお気軽にご来店いただけます！！
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>26724</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>21:33:39</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>きんたまよ</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2人でデート帰り</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>ギンギンと雨でびしゃびしゃもう着きます</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>26725</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>21:35:58</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ゆずき</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>仕事終わりに</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>きました！！</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>26726</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>21:36:28</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>26727</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>21:36:39</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>26728</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>21:51:29</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>マロ</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>久しぶりに</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>エルちゃんに会いに！</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>26729</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>22:41:17</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>のり、あや</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ふたりで</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>きたよー！！</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>26730</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>22:43:44</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ひろとも、ゆうき</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>はじめて</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>気になってきちゃいました♪</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>26731</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>22:44:01</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>26732</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>22:44:17</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>26733</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>22:44:28</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>26734</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>00:43:48</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>テクノとポチ</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ふたりで</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>きまちた♪</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>26735</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>00:44:18</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>26736</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>01:16:21</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>まいまい</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>少し休んでから</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>きた！</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>26737</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>01:20:38</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>26738</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>03:46:49</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>JPTR</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>みんなで</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>はじめてきました！</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>26739</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>03:55:48</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>26741</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>04:29:59</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの水曜日営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>本日8月11日の営業時間は♪
+オープン14:00！ラスト5:00なのよ☆
+担当は
+ツッコミはお任せのShizu
+えちえち裏垢女子のモカチ
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>img20260812042959.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>26742</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>04:31:31</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>☆割引キャンペーン開催中☆</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>【団体割引キャンペーン見ました】と
+受付スタッフに言って頂ければ…
+／
+おひとり様毎に！！
+2000円割引します！！！
+＼
+お得に遊びませんか？
+仕事終わり、飲み会終わりなど
+ぜひぜひお気軽にお越しくださいませ♪
+【団体割引キャンペーン見ました】と
+受付スタッフに言って頂ければ…
+／
+おひとり様毎に！！
+2000円割引します！！！
+＼
+お得に遊びませんか？
+仕事終わり、飲み会終わりなど
+ぜひぜひお気軽にお越しくださいませ♪</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>img20260812043131.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: BBS取得 2026-08-12 22:59 UTC
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2318,7 +2318,6 @@
 本日、伺います</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2352,7 +2351,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2383,7 +2381,6 @@
           <t>きてます！！</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2416,7 +2413,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2447,7 +2443,6 @@
           <t>緊張しますが行ってみようと思います！</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2481,7 +2476,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2512,7 +2506,6 @@
           <t>ギンギンと雨でびしゃびしゃもう着きます</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2543,7 +2536,6 @@
           <t>きました！！</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2576,7 +2568,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2609,7 +2600,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2640,7 +2630,6 @@
           <t>エルちゃんに会いに！</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2671,7 +2660,6 @@
           <t>きたよー！！</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2702,7 +2690,6 @@
           <t>気になってきちゃいました♪</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2735,7 +2722,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2768,7 +2754,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2801,7 +2786,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2832,7 +2816,6 @@
           <t>きまちた♪</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2865,7 +2848,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2896,7 +2878,6 @@
           <t>きた！</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2929,7 +2910,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2960,7 +2940,6 @@
           <t>はじめてきました！</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2993,7 +2972,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3095,6 +3073,1257 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>26743</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>14:54:08</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ゆぴ</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>連休</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>楽しみます</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>26744</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>15:14:31</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>26745</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>17:37:22</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ゆずき</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>連日</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>登場！</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>26746</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>17:39:06</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>マッスル</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>こんちわ</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>きまっする</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>26747</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>17:39:40</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>26748</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>17:39:51</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>26749</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>19:11:18</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>やえ</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>都内かえり</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>26750</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>19:12:18</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>かずき、フジ</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>二人で</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>二年ぶり</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>26751</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>19:13:57</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>26752</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>19:14:09</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>26753</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>ゆうき</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>ひさしぶり</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>26754</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>20:39:19</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>26755</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>21:13:40</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>よしおたん</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>韓国パブ</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>いってきた</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>26756</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>21:13:57</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>26757</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>21:37:26</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>りゅう、たく</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>26758</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>21:38:52</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>26759</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>21:52:18</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>きちゃ！</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>26760</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>21:52:35</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>よしやん、かな</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>きまんた</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>26761</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>26762</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>21:53:11</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>26763</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>23:13:38</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>マナティ</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>酔い冷ましに</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>行きます</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>26764</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>23:14:29</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>26765</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>01:39:12</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>あゆ</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>26766</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>01:46:01</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>げん、ともち</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>26767</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>01:46:28</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>26768</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>01:46:39</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>26769</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>02:07:49</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>まおし</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>ひさびさに</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>きたゆ</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>26770</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>02:08:11</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>26771</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>02:37:55</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>すー</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>きちゃ</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>26772</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>02:38:15</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>26773</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>02:55:31</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>たかやま、りりこ</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>きた！</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>26774</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>02:55:54</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>まいまいん</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>きちゃー！！！！</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>26775</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>02:56:22</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>26776</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>02:56:33</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>26777</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>03:20:48</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>キム、みれい</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>さっき</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>きまちた</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>26778</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>03:44:47</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>26779</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>03:49:01</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの木曜日営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>本日8月13日の営業時間は♪
+オープン19:00！ラスト5:00なのよ☆
+担当は
+ツッコミはお任せのShizu
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>img20260813034901.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>26780</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>03:49:54</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>☆割引キャンペーン開催中☆</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>【団体割引キャンペーン見ました】と
+受付スタッフに言って頂ければ…
+／
+おひとり様毎に！！
+2000円割引します！！！
+＼
+お得に遊びませんか？
+仕事終わり、飲み会終わりなど
+ぜひぜひお気軽にお越しくださいませ♪
+【団体割引キャンペーン見ました】と
+受付スタッフに言って頂ければ…
+／
+おひとり様毎に！！
+2000円割引します！！！
+＼
+お得に遊びませんか？
+仕事終わり、飲み会終わりなど
+ぜひぜひお気軽にお越しくださいませ♪</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>img20260813034954.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: BBS取得 2026-08-13 23:00 UTC
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3102,7 +3102,6 @@
           <t>楽しみます</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3135,7 +3134,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3166,7 +3164,6 @@
           <t>登場！</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3197,7 +3194,6 @@
           <t>きまっする</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3230,7 +3226,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3263,7 +3258,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3294,7 +3288,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3325,7 +3318,6 @@
           <t>二年ぶり</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3358,7 +3350,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3391,7 +3382,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3422,7 +3412,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3455,7 +3444,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3486,7 +3474,6 @@
           <t>いってきた</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3519,7 +3506,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3550,7 +3536,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3583,7 +3568,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3614,7 +3598,6 @@
           <t>きちゃ！</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3645,7 +3628,6 @@
           <t>きまんた</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3678,7 +3660,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3711,7 +3692,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3742,7 +3722,6 @@
           <t>行きます</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -3775,7 +3754,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -3806,7 +3784,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -3837,7 +3814,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -3870,7 +3846,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -3903,7 +3878,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -3934,7 +3908,6 @@
           <t>きたゆ</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -3967,7 +3940,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -3998,7 +3970,6 @@
           <t>きちゃ</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -4031,7 +4002,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -4062,7 +4032,6 @@
           <t>きた！</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -4093,7 +4062,6 @@
           <t>きちゃー！！！！</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -4126,7 +4094,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -4159,7 +4126,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -4190,7 +4156,6 @@
           <t>きまちた</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -4223,7 +4188,6 @@
 スタッフ一同心よりお待ちしておりますね♪</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -4324,6 +4288,1066 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>26781</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>19:10:31</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>ふみ</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>はじめて</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>きました♪</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>26782</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>19:11:47</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>26783</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>19:16:23</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>ほぼ</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>オープン凸</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>26784</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>19:16:46</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>26785</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>のんのん</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>めずらしく</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>はやめに！</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>26786</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>20:08:06</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>きむ、りさ</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>今日も</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>26787</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>20:10:37</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>りん</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>飲みに</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>26788</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>20:10:59</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>26789</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>20:11:23</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>26790</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>20:11:42</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>26791</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>20:24:38</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>たます</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>ひさしぶり</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>26792</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>20:24:51</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>26793</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>21:05:25</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>かける</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>はじめて</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>26794</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>21:05:39</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>26795</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>21:27:52</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>オ・スー</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>あそびに</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>きましたよ</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>26796</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>21:28:08</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>26797</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>23:31:30</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>ぽちゃりす組</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>いま</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>26798</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>23:31:45</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>26799</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>01:11:19</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>おちんぽベルセルク</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>すこし</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>きました♪</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>26800</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>01:11:39</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>26801</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>01:31:53</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>zin、あゆ</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>仕事終わりに</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>26802</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>01:32:22</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>26803</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>01:34:21</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>みれい</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>昨日ぶり</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>26804</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>01:34:41</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>26805</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>02:06:00</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>ごん、ぶりちゃん</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>二人で</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>26806</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>02:06:19</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>26807</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>02:20:44</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>まい</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>シゴオワ</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>きた</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>26808</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>02:21:07</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>TKC</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>飲みに</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>きた！</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>26809</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>02:21:24</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>おぉぉぉぉぉぉぉぉぉ♪</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>26810</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>02:21:34</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>お待ちしておりまぁす♪</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>来店予告ありがとうございます♪
+ぜひぜひお越し下さい☆
+スタッフ一同心よりお待ちしておりますね♪</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>26811</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>04:24:18</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの週末営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>本日8月14日の営業時間は♪
+オープン19:00！ラスト5:00なのよ☆
+担当は
+ツッコミはお任せのShizu
+新妻マゾヒストのミコト
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>img20260814042418.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>26812</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>04:26:24</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>☆割引キャンペーン開催中☆</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>【団体割引キャンペーン見ました】と
+受付スタッフに言って頂ければ…
+／
+おひとり様毎に！！
+2000円割引します！！！
+＼
+お得に遊びませんか？
+仕事終わり、飲み会終わりなど
+ぜひぜひお気軽にお越しくださいませ♪
+【団体割引キャンペーン見ました】と
+受付スタッフに言って頂ければ…
+／
+おひとり様毎に！！
+2000円割引します！！！
+＼
+お得に遊びませんか？
+仕事終わり、飲み会終わりなど
+ぜひぜひお気軽にお越しくださいませ♪</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>img20260814042624.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: BBS取得 2026-08-14 22:38 UTC
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,7 +477,6 @@
           <t>いぬ、マッチョ、ももたろ</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>ムキムキ三人衆で</t>
@@ -508,7 +507,6 @@
           <t>ゆうたん、カモリ</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>カップルで</t>
@@ -539,7 +537,6 @@
           <t>アキ、コオリ</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>はじめてさん連れて</t>
@@ -570,7 +567,6 @@
           <t>ゆずき</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>ちょいのみ</t>
@@ -601,7 +597,6 @@
           <t>てつ</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>田中</t>
@@ -632,7 +627,6 @@
           <t>H,M,D</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>みんなで</t>
@@ -663,7 +657,6 @@
           <t>ともゆき</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -694,7 +687,6 @@
           <t>まいまい</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>しごわ</t>
@@ -777,7 +769,6 @@
           <t>はなまる</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>久しぶりの</t>
@@ -808,7 +799,6 @@
           <t>大塚</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>今</t>
@@ -839,7 +829,6 @@
           <t>ゆうと</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -870,7 +859,6 @@
           <t>カー</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>今</t>
@@ -901,7 +889,6 @@
           <t>ミコト、まいまい、テクノ</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>ちいかわ</t>
@@ -932,7 +919,6 @@
           <t>りょうちゃん</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>バンビ</t>
@@ -963,7 +949,6 @@
           <t>らうら</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>少し</t>
@@ -994,7 +979,6 @@
           <t>タツヤ</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>牛タン青味噌</t>
@@ -1025,7 +1009,6 @@
           <t>ふくてゃ、T山</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>激辛祭り！</t>
@@ -1056,7 +1039,6 @@
           <t>ひがん</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>イベたのしみに</t>
@@ -1087,7 +1069,6 @@
           <t>Bee</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>今週も</t>
@@ -1118,7 +1099,6 @@
           <t>−、N</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>辛いの苦手だけど</t>
@@ -1149,7 +1129,6 @@
           <t>テクノ</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>麻婆豆腐</t>
@@ -1180,7 +1159,6 @@
           <t>KUMA</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>大宮バンビから</t>
@@ -1211,7 +1189,6 @@
           <t>コテッチャン</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>来たぜ</t>
@@ -1242,7 +1219,6 @@
           <t>なお</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>お土産</t>
@@ -1273,7 +1249,6 @@
           <t>ボンタ</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -1304,7 +1279,6 @@
           <t>ゆん</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>久々</t>
@@ -1335,7 +1309,6 @@
           <t>でで</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>イベ楽しみに</t>
@@ -1366,7 +1339,6 @@
           <t>いっちゃん</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>遊びに</t>
@@ -1397,7 +1369,6 @@
           <t>だいち</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>初来店</t>
@@ -1429,7 +1400,6 @@
           <t>ダイチ</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -1460,7 +1430,6 @@
           <t>nuri</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>はじめていきます</t>
@@ -1491,7 +1460,6 @@
           <t>きんたまよ</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>2人でデート帰り</t>
@@ -1522,7 +1490,6 @@
           <t>ゆずき</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>仕事終わりに</t>
@@ -1553,7 +1520,6 @@
           <t>マロ</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>久しぶりに</t>
@@ -1584,7 +1550,6 @@
           <t>のり、あや</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>ふたりで</t>
@@ -1615,7 +1580,6 @@
           <t>ひろとも、ゆうき</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -1646,7 +1610,6 @@
           <t>テクノとポチ</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>ふたりで</t>
@@ -1677,7 +1640,6 @@
           <t>まいまい</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>少し休んでから</t>
@@ -1708,7 +1670,6 @@
           <t>JPTR</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>みんなで</t>
@@ -1792,7 +1753,6 @@
           <t>ゆぴ</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>連休</t>
@@ -1823,7 +1783,6 @@
           <t>ゆずき</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>連日</t>
@@ -1854,7 +1813,6 @@
           <t>マッスル</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>こんちわ</t>
@@ -1885,7 +1843,6 @@
           <t>やえ</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>都内かえり</t>
@@ -1916,7 +1873,6 @@
           <t>かずき、フジ</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>二人で</t>
@@ -1947,7 +1903,6 @@
           <t>ゆうき</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>ひさしぶり</t>
@@ -1978,7 +1933,6 @@
           <t>よしおたん</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>韓国パブ</t>
@@ -2009,7 +1963,6 @@
           <t>りゅう、たく</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>今</t>
@@ -2040,7 +1993,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>今</t>
@@ -2071,7 +2023,6 @@
           <t>よしやん、かな</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>今</t>
@@ -2102,7 +2053,6 @@
           <t>マナティ</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>酔い冷ましに</t>
@@ -2133,7 +2083,6 @@
           <t>あゆ</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>今</t>
@@ -2164,7 +2113,6 @@
           <t>げん、ともち</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>今</t>
@@ -2195,7 +2143,6 @@
           <t>まおし</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>ひさびさに</t>
@@ -2226,7 +2173,6 @@
           <t>すー</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>今</t>
@@ -2257,7 +2203,6 @@
           <t>たかやま、りりこ</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>今</t>
@@ -2288,7 +2233,6 @@
           <t>まいまいん</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>今</t>
@@ -2319,7 +2263,6 @@
           <t>キム、みれい</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>さっき</t>
@@ -2402,7 +2345,6 @@
           <t>ふみ</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -2433,7 +2375,6 @@
           <t>ひがん</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>ほぼ</t>
@@ -2464,7 +2405,6 @@
           <t>のんのん</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>めずらしく</t>
@@ -2495,7 +2435,6 @@
           <t>きむ、りさ</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>今日も</t>
@@ -2526,7 +2465,6 @@
           <t>りん</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>飲みに</t>
@@ -2557,7 +2495,6 @@
           <t>たます</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>ひさしぶり</t>
@@ -2588,7 +2525,6 @@
           <t>かける</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -2619,7 +2555,6 @@
           <t>オ・スー</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>あそびに</t>
@@ -2650,7 +2585,6 @@
           <t>ぽちゃりす組</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>いま</t>
@@ -2681,7 +2615,6 @@
           <t>おちんぽベルセルク</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>すこし</t>
@@ -2712,7 +2645,6 @@
           <t>zin、あゆ</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>仕事終わりに</t>
@@ -2743,7 +2675,6 @@
           <t>みれい</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>昨日ぶり</t>
@@ -2774,7 +2705,6 @@
           <t>ごん、ぶりちゃん</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>二人で</t>
@@ -2805,7 +2735,6 @@
           <t>まい</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>シゴオワ</t>
@@ -2836,7 +2765,6 @@
           <t>TKC</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>飲みに</t>
@@ -2901,6 +2829,827 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>26813</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>19:06:50</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>おとは</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>金曜</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>きたよーん♪</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>26814</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>19:07:26</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>よっち</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>今日はオープンから</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>26817</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>19:24:35</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>りょう</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>これから</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>これから寄ってみます！</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>26818</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>19:32:01</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>まいまい、ゆずき</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>飲みおわ</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>きました！！</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>26819</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>19:40:45</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>マッスル</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>今日も</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>きまんた！</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>26820</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>19:43:56</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ねここ</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>はじめて</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>26821</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>19:51:19</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ゆず、ちぇちぇ</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>はじめて二人で</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>きました！！</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>26822</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>20:15:26</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>たいせー</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>緊張しますが、本日お伺いします</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>26823</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>20:18:29</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>bee</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>ぶんぶん</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>蜂さん！</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>26824</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>20:18:55</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>カズ</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>今日は</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>早めに来ました</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>26833</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>21:45:29</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>たいせい</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>来ました！！</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>26834</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>21:48:50</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>かい</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>前橋から</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>来ました！！</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>26837</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>21:58:15</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>るい</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>26838</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>22:05:09</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>タツヤ</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>戦って</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>きましたー</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>26839</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>22:06:17</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>ででたゃ</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>きたよん！</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>26843</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>22:48:24</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>あにー、りえ、ゆり</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>しごおわ</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>行くマス</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>26845</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>22:55:59</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>みなっち</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>26849</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>23:22:10</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>しゅん</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>いきます</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>久しぶりに</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>26851</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>00:11:14</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>きむら</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>今から</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>おじやましますー</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>26853</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>00:13:48</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>いま</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>26855</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>00:44:59</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>ましゅ、絶</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>26857</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>01:35:32</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>りお、めい、まい</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>しごおわ</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>26859</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>02:19:37</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>だいご</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>よばれて</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>きちゃよ</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>26861</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>02:59:37</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>ザッキー、よっしー</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>きました♪</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>26863</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>03:58:08</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>ツッコミはお任せのShizu / えちえち裏垢女子のモカチ</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの週末営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>本日8月15日の営業時間は♪
+オープン19:00！ラスト5:00なのよ☆
+担当は
+ツッコミはお任せのShizu
+えちえち裏垢女子のモカチ
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>img20260815035808.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: BBS取得 2026-08-15 22:36 UTC
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2848,7 +2848,6 @@
           <t>おとは</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>金曜</t>
@@ -2859,7 +2858,6 @@
           <t>きたよーん♪</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2880,7 +2878,6 @@
           <t>よっち</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>今日はオープンから</t>
@@ -2891,7 +2888,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2912,7 +2908,6 @@
           <t>りょう</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>これから</t>
@@ -2923,7 +2918,6 @@
           <t>これから寄ってみます！</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2944,7 +2938,6 @@
           <t>まいまい、ゆずき</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>飲みおわ</t>
@@ -2955,7 +2948,6 @@
           <t>きました！！</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2976,7 +2968,6 @@
           <t>マッスル</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>今日も</t>
@@ -2987,7 +2978,6 @@
           <t>きまんた！</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3008,7 +2998,6 @@
           <t>ねここ</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -3019,7 +3008,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3040,7 +3028,6 @@
           <t>ゆず、ちぇちぇ</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>はじめて二人で</t>
@@ -3051,7 +3038,6 @@
           <t>きました！！</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3072,7 +3058,6 @@
           <t>たいせー</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -3083,7 +3068,6 @@
           <t>緊張しますが、本日お伺いします</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3104,7 +3088,6 @@
           <t>bee</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>ぶんぶん</t>
@@ -3115,7 +3098,6 @@
           <t>蜂さん！</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3136,7 +3118,6 @@
           <t>カズ</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>今日は</t>
@@ -3147,7 +3128,6 @@
           <t>早めに来ました</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3168,7 +3148,6 @@
           <t>たいせい</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -3179,7 +3158,6 @@
           <t>来ました！！</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3200,7 +3178,6 @@
           <t>かい</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>前橋から</t>
@@ -3211,7 +3188,6 @@
           <t>来ました！！</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3232,7 +3208,6 @@
           <t>るい</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>遊びに</t>
@@ -3243,7 +3218,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3264,7 +3238,6 @@
           <t>タツヤ</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>戦って</t>
@@ -3275,7 +3248,6 @@
           <t>きましたー</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3296,7 +3268,6 @@
           <t>ででたゃ</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>遊びに</t>
@@ -3307,7 +3278,6 @@
           <t>きたよん！</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3328,7 +3298,6 @@
           <t>あにー、りえ、ゆり</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>しごおわ</t>
@@ -3339,7 +3308,6 @@
           <t>行くマス</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3360,7 +3328,6 @@
           <t>みなっち</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>遊びに</t>
@@ -3371,7 +3338,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3392,7 +3358,6 @@
           <t>しゅん</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>いきます</t>
@@ -3403,7 +3368,6 @@
           <t>久しぶりに</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3424,7 +3388,6 @@
           <t>きむら</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>今から</t>
@@ -3435,7 +3398,6 @@
           <t>おじやましますー</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3456,7 +3418,6 @@
           <t>ひがん</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>いま</t>
@@ -3467,7 +3428,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3488,7 +3448,6 @@
           <t>ましゅ、絶</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>遊びに</t>
@@ -3499,7 +3458,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3520,7 +3478,6 @@
           <t>りお、めい、まい</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>しごおわ</t>
@@ -3531,7 +3488,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3552,7 +3508,6 @@
           <t>だいご</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>よばれて</t>
@@ -3563,7 +3518,6 @@
           <t>きちゃよ</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3584,7 +3538,6 @@
           <t>ザッキー、よっしー</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -3595,7 +3548,6 @@
           <t>きました♪</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3650,6 +3602,826 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>26865</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>18:51:45</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>おじきち</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>きたよ！</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>26867</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>18:57:32</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>まろ、おとは</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>はやめに</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>きたよ</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>26869</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>19:28:11</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>たつや</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>きたｚ</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>26870</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>19:28:38</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>S、Y</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>２回目</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>26871</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>19:28:53</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>よっち</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>26875</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>19:49:47</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ゆずき</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>きょうも</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>いるよ</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>26876</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>19:50:08</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>まっする</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>きたんご</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>26879</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>20:30:43</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>26881</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>20:46:17</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>まいなちゅ、えぬ</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>きちゃ</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>26882</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>20:46:44</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>こてっちゃん</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>ひさびさ土曜に</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>きたよ！</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>26885</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>21:38:55</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>みーみ</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>ひさびさ</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>26887</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>22:17:43</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>あっくん、まりん</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>ひさしぶり</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>きました♪</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>26889</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>22:48:19</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>いま</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>お土産持ってきた！</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>26891</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>23:09:30</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>NMGK、彩</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>二人で</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>26893</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>23:14:42</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>だいさく、たくや</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>今日は</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>ふたりで！</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>26895</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>ましゅ、きむ、どえむちゃん</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>三人で</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>26897</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>00:42:06</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>女子三人衆</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>きました！！</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>26898</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>00:42:29</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>かず、のんのん</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>さっき</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>きたよ</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>26899</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>00:42:42</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>けん</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>初めて</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>きました</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>26903</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>01:04:50</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>れー、ぷらぐいん</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>今</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>きまいた</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>26905</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>01:31:58</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>K、N</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>今日も</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>きたよ！</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>26906</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>01:32:06</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>ぺぺ</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>このあといきます！</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>初めまして、よろしくお願いします！</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>26907</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>01:32:29</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>みずき、りく、りん</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>女子三人</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>26911</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>02:19:30</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>しん</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>いま</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>きたんご</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>26913</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>04:06:23</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>天然の100人ネキのねむ</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの日曜日営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>本日8月16日の営業時間は♪
+オープン19:00！ラスト5:00なのよ☆
+担当は
+天然の100人ネキのねむ
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>img20260816040623.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: BBS取得 2026-08-17 22:38 UTC
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H144"/>
+  <dimension ref="A1:H154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4399,7 +4399,6 @@
           <t>たいせい</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>2回目</t>
@@ -4410,7 +4409,6 @@
           <t>きたよ</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -4431,7 +4429,6 @@
           <t>ひがん</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>オープン凸</t>
@@ -4442,7 +4439,6 @@
           <t>きた</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -4463,7 +4459,6 @@
           <t>くま、まーくん、とおちゃん</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>3人で</t>
@@ -4474,7 +4469,6 @@
           <t>初めて</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -4495,7 +4489,6 @@
           <t>みかん</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>もうちょっと</t>
@@ -4506,7 +4499,6 @@
           <t>あと少しで行きます</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -4527,7 +4519,6 @@
           <t>なお</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>すこし</t>
@@ -4538,7 +4529,6 @@
           <t>きたよ</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -4559,7 +4549,6 @@
           <t>ナカヤマヤ</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>ずっと</t>
@@ -4570,7 +4559,6 @@
           <t>気になってて</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -4591,7 +4579,6 @@
           <t>しーたん</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>今から行きます</t>
@@ -4602,7 +4589,6 @@
           <t>お願い致します</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -4623,7 +4609,6 @@
           <t>みなつちん</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>後半に入って仕事終わってから</t>
@@ -4634,7 +4619,6 @@
           <t>いぐぅぅ</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -4655,7 +4639,6 @@
           <t>テクノ</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>今日は</t>
@@ -4666,7 +4649,6 @@
           <t>フリーで</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -4687,7 +4669,6 @@
           <t>キムと奴隷</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>今日も</t>
@@ -4698,7 +4679,6 @@
           <t>来店します</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -4719,7 +4699,6 @@
           <t>すーたく、ことり</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>いま</t>
@@ -4730,7 +4709,6 @@
           <t>きたでー</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -4751,7 +4729,6 @@
           <t>マイナス</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>今</t>
@@ -4762,7 +4739,6 @@
           <t>きたった</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -4783,7 +4759,6 @@
           <t>すず</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>横浜から</t>
@@ -4794,7 +4769,6 @@
           <t>お初</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -4815,7 +4789,6 @@
           <t>ゆきんこ、いぬ、てっちゃん、ながとも</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>みんなで</t>
@@ -4826,7 +4799,6 @@
           <t>きたぜ</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -4847,7 +4819,6 @@
           <t>ゆうくん</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>呼ばれて</t>
@@ -4858,7 +4829,6 @@
           <t>きたよー</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -4879,7 +4849,6 @@
           <t>みなっち</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>ただいま</t>
@@ -4890,7 +4859,6 @@
           <t>参上</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -4944,6 +4912,346 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>26951</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>19:21:57</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>まいなす</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>早めに</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>来たよー♪</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>26953</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>19:44:27</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>なお</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>今日は</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>長めにいますー</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>26955</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>20:02:03</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>あや</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>きたよ！</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>26956</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>20:03:40</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>たかやま</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>今日は夜まで</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>のんびりと</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>26959</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>21:07:46</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>にこちん</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>11時頃</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>目標に行きます。</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>26961</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>23:42:16</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>れいら</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>しごおわ</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>来たよー</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>26963</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>23:57:47</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>さくら</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>きましたー！</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>26964</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>23:58:16</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>zin</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>ちょい</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>26965</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>01:54:10</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>すーさん</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>来たぜ</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>26969</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>03:32:35</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>天然の100人ネキ　ねむ</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの火曜日営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>本日8月17日の営業時間は♪
+オープン19:00！ラスト5:00なのよ☆
+担当は
+天然の100人ネキ　ねむ
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>img20260818033235.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4955,7 +5263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I185"/>
+  <dimension ref="A1:I194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12915,6 +13223,393 @@
       <c r="I185" t="inlineStr">
         <is>
           <t>参上</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>19:21:57</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>26951</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>まいなす</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>1</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>まいなす</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>早めに</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>来たよー♪</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>19:44:27</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>26953</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>なお</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>3</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>なお</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>今日は</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>長めにいますー</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>20:02:03</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>26955</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>あや</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>2</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>あや</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>きたよ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>20:03:40</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>26956</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>たかやま</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>2</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>たかやま</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>今日は夜まで</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>のんびりと</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>21:07:46</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>26959</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>にこちん</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>1</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>にこちん</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>11時頃</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>目標に行きます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>23:42:16</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>26961</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>れいら</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>1</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>れいら</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>しごおわ</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>来たよー</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>23:57:47</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>26963</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>さくら</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>1</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>さくら</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>きましたー！</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>23:58:16</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>26964</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>zin</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>2</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>zin</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>ちょい</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>きました！</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>01:54:10</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>26965</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>すーさん</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>1</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>すーさん</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>来たぜ</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>遊びに</t>
         </is>
       </c>
     </row>
@@ -12929,7 +13624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D155"/>
+  <dimension ref="A1:D160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13017,7 +13712,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>テクノ</t>
+          <t>なお</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -13025,27 +13720,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>テクノ</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -13057,7 +13752,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>あゆ</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -13065,19 +13760,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>いぬ</t>
+          <t>zin</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -13085,7 +13780,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -13097,7 +13792,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>おとは</t>
+          <t>あや</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -13105,19 +13800,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>きむ</t>
+          <t>あゆ</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -13130,14 +13825,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>たいせい</t>
+          <t>いぬ</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -13145,19 +13840,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>なお</t>
+          <t>おとは</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -13165,19 +13860,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>のんのん</t>
+          <t>きむ</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -13197,7 +13892,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>まい</t>
+          <t>たいせい</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -13210,14 +13905,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ましゅ</t>
+          <t>たかやま</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -13225,19 +13920,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>みなっち</t>
+          <t>のんのん</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -13245,19 +13940,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>みれい</t>
+          <t>まい</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -13265,19 +13960,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ゆうき</t>
+          <t>ましゅ</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -13285,19 +13980,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>よっち</t>
+          <t>みなっち</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -13310,14 +14005,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>りん</t>
+          <t>みれい</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -13330,14 +14025,14 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>タツヤ</t>
+          <t>ゆうき</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -13345,19 +14040,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>マッスル</t>
+          <t>よっち</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -13365,43 +14060,43 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>りん</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bee</t>
+          <t>タツヤ</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -13410,34 +14105,34 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>マッスル</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -13445,19 +14140,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>JPTR</t>
+          <t>Bee</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -13465,19 +14160,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -13485,19 +14180,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>KUMA</t>
+          <t>H</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -13505,19 +14200,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>JPTR</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -13525,19 +14220,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NMGK</t>
+          <t>K</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -13545,19 +14240,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>KUMA</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -13565,19 +14260,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>STR</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -13585,19 +14280,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TKC</t>
+          <t>NMGK</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -13605,19 +14300,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>T山</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -13625,19 +14320,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -13657,7 +14352,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>bee</t>
+          <t>TKC</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -13677,7 +14372,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>nuri</t>
+          <t>T山</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -13685,19 +14380,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>zin</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -13705,19 +14400,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>−</t>
+          <t>bee</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -13725,19 +14420,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>あっくん</t>
+          <t>nuri</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -13745,19 +14440,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>あにー</t>
+          <t>−</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -13765,19 +14460,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>あや</t>
+          <t>あっくん</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -13785,19 +14480,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>いっちゃん</t>
+          <t>あにー</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -13805,19 +14500,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>えぬ</t>
+          <t>いっちゃん</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -13825,19 +14520,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>おじきち</t>
+          <t>えぬ</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -13857,7 +14552,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>おちんぽベルセルク</t>
+          <t>おじきち</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -13865,19 +14560,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>かい</t>
+          <t>おちんぽベルセルク</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -13897,7 +14592,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>かける</t>
+          <t>かい</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -13905,19 +14600,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>かず</t>
+          <t>かける</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -13925,19 +14620,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>かずき</t>
+          <t>かず</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -13945,19 +14640,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>かな</t>
+          <t>かずき</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -13977,7 +14672,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>きむら</t>
+          <t>かな</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -13985,19 +14680,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>きんたまよ</t>
+          <t>きむら</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -14005,19 +14700,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>くま</t>
+          <t>きんたまよ</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -14025,19 +14720,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>けん</t>
+          <t>くま</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -14057,7 +14752,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>げん</t>
+          <t>けん</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -14065,19 +14760,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>こてっちゃん</t>
+          <t>げん</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -14085,19 +14780,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ことり</t>
+          <t>こてっちゃん</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -14105,19 +14800,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ごん</t>
+          <t>ことり</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -14125,19 +14820,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>しゅん</t>
+          <t>ごん</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -14157,7 +14852,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>しん</t>
+          <t>さくら</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -14165,19 +14860,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>しーたん</t>
+          <t>しゅん</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -14185,19 +14880,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>すず</t>
+          <t>しん</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -14217,7 +14912,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>すー</t>
+          <t>しーたん</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -14225,19 +14920,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>すーたく</t>
+          <t>すず</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -14257,7 +14952,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>たいせー</t>
+          <t>すー</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -14265,19 +14960,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>たかやま</t>
+          <t>すーさん</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -14285,19 +14980,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>たく</t>
+          <t>すーたく</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -14305,19 +15000,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>たくや</t>
+          <t>たいせー</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -14325,19 +15020,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>たつや</t>
+          <t>たく</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -14345,19 +15040,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>たます</t>
+          <t>たくや</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -14365,19 +15060,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>だいご</t>
+          <t>たつや</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -14397,7 +15092,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>だいさく</t>
+          <t>たます</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -14405,19 +15100,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>だいち</t>
+          <t>だいご</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -14425,19 +15120,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ちぇちぇ</t>
+          <t>だいさく</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -14445,19 +15140,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>てっちゃん</t>
+          <t>だいち</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -14465,19 +15160,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>てつ</t>
+          <t>ちぇちぇ</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -14485,19 +15180,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>でで</t>
+          <t>てっちゃん</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -14505,19 +15200,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ででたゃ</t>
+          <t>てつ</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -14525,19 +15220,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>とおちゃん</t>
+          <t>でで</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -14545,19 +15240,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ともち</t>
+          <t>ででたゃ</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -14565,19 +15260,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ともゆき</t>
+          <t>とおちゃん</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -14585,19 +15280,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>どえむちゃん</t>
+          <t>ともち</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -14605,19 +15300,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ながとも</t>
+          <t>ともゆき</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -14625,19 +15320,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ねここ</t>
+          <t>どえむちゃん</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -14645,19 +15340,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>のり</t>
+          <t>ながとも</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -14665,19 +15360,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>はなまる</t>
+          <t>にこちん</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -14685,19 +15380,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ひろとも</t>
+          <t>ねここ</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -14705,19 +15400,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ふくてゃ</t>
+          <t>のり</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -14725,19 +15420,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ふみ</t>
+          <t>はなまる</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -14745,19 +15440,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ぶりちゃん</t>
+          <t>ひろとも</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -14765,19 +15460,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ぷらぐいん</t>
+          <t>ふくてゃ</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -14785,19 +15480,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ぺぺ</t>
+          <t>ふみ</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -14805,19 +15500,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ぽちゃりす組</t>
+          <t>ぶりちゃん</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -14825,19 +15520,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>まいなちゅ</t>
+          <t>ぷらぐいん</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -14845,19 +15540,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>まいまいん</t>
+          <t>ぺぺ</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -14865,19 +15560,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>まおし</t>
+          <t>ぽちゃりす組</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -14897,7 +15592,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>まっする</t>
+          <t>まいなす</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -14905,19 +15600,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>まりん</t>
+          <t>まいなちゅ</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -14937,7 +15632,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>まろ</t>
+          <t>まいまいん</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -14945,19 +15640,19 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>まーくん</t>
+          <t>まおし</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -14965,19 +15660,19 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>みかん</t>
+          <t>まっする</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -14985,19 +15680,19 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>みずき</t>
+          <t>まりん</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -15005,19 +15700,19 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>みなつちん</t>
+          <t>まろ</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -15025,19 +15720,19 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>みーみ</t>
+          <t>まーくん</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -15045,19 +15740,19 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>めい</t>
+          <t>みかん</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -15065,19 +15760,19 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ももたろ</t>
+          <t>みずき</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -15085,19 +15780,19 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>やえ</t>
+          <t>みなつちん</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -15105,19 +15800,19 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ゆうくん</t>
+          <t>みーみ</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -15125,19 +15820,19 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ゆうたん</t>
+          <t>めい</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -15145,19 +15840,19 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ゆうと</t>
+          <t>ももたろ</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -15165,19 +15860,19 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ゆきんこ</t>
+          <t>やえ</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -15185,19 +15880,19 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ゆず</t>
+          <t>ゆうくん</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -15205,19 +15900,19 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ゆぴ</t>
+          <t>ゆうたん</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -15225,19 +15920,19 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ゆり</t>
+          <t>ゆうと</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -15245,19 +15940,19 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ゆん</t>
+          <t>ゆきんこ</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -15265,19 +15960,19 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>よしおたん</t>
+          <t>ゆず</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -15285,19 +15980,19 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>よしやん</t>
+          <t>ゆぴ</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -15317,7 +16012,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>よっしー</t>
+          <t>ゆり</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -15325,19 +16020,19 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>らうら</t>
+          <t>ゆん</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -15357,7 +16052,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>りえ</t>
+          <t>よしおたん</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -15365,19 +16060,19 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>りお</t>
+          <t>よしやん</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -15385,19 +16080,19 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>りく</t>
+          <t>よっしー</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -15405,19 +16100,19 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>りさ</t>
+          <t>らうら</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -15425,19 +16120,19 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>りゅう</t>
+          <t>りえ</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -15445,19 +16140,19 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>りょう</t>
+          <t>りお</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -15465,19 +16160,19 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>りょうちゃん</t>
+          <t>りく</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -15485,19 +16180,19 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>りりこ</t>
+          <t>りさ</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -15517,7 +16212,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>るい</t>
+          <t>りゅう</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -15525,19 +16220,19 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>れー</t>
+          <t>りょう</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -15545,19 +16240,19 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>アキ</t>
+          <t>りょうちゃん</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -15565,19 +16260,19 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>オ・スー</t>
+          <t>りりこ</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -15597,7 +16292,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>カズ</t>
+          <t>るい</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -15617,7 +16312,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>カモリ</t>
+          <t>れいら</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -15625,19 +16320,19 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>カー</t>
+          <t>れー</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -15645,19 +16340,19 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>キム</t>
+          <t>アキ</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -15665,19 +16360,19 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>キムと奴隷</t>
+          <t>オ・スー</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -15685,19 +16380,19 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>コオリ</t>
+          <t>カズ</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -15705,19 +16400,19 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>コテッチャン</t>
+          <t>カモリ</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -15737,7 +16432,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ザッキー</t>
+          <t>カー</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -15745,19 +16440,19 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ダイチ</t>
+          <t>キム</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -15765,19 +16460,19 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>テクノとポチ</t>
+          <t>キムと奴隷</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -15785,19 +16480,19 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ナカヤマヤ</t>
+          <t>コオリ</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -15805,19 +16500,19 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>フジ</t>
+          <t>コテッチャン</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -15825,19 +16520,19 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ボンタ</t>
+          <t>ザッキー</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -15845,19 +16540,19 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>マイナス</t>
+          <t>ダイチ</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -15865,19 +16560,19 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>マッチョ</t>
+          <t>テクノとポチ</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -15885,19 +16580,19 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>マナティ</t>
+          <t>ナカヤマヤ</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -15905,19 +16600,19 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>マロ</t>
+          <t>フジ</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -15925,19 +16620,19 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ミコト</t>
+          <t>ボンタ</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -15945,19 +16640,19 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>大塚</t>
+          <t>マイナス</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -15965,19 +16660,19 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>女子三人衆</t>
+          <t>マッチョ</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -15985,19 +16680,19 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>彩</t>
+          <t>マナティ</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -16005,30 +16700,130 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
+          <t>マロ</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>ミコト</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>大塚</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>女子三人衆</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>彩</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
           <t>絶</t>
         </is>
       </c>
-      <c r="B155" t="n">
-        <v>1</v>
-      </c>
-      <c r="C155" t="inlineStr">
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr">
+      <c r="D160" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
@@ -16072,10 +16867,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -16085,10 +16880,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -16207,10 +17002,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -16441,10 +17236,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C21" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22">
@@ -16454,10 +17249,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C22" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23">
@@ -16467,10 +17262,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24">
@@ -16493,10 +17288,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C25" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -16542,13 +17337,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="C2" t="n">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="D2" t="n">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: BBS取得 2026-09-01 01:16 UTC
</commit_message>
<xml_diff>
--- a/bbs_log.xlsx
+++ b/bbs_log.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H346"/>
+  <dimension ref="A1:H353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10423,7 +10423,6 @@
           <t>すず</t>
         </is>
       </c>
-      <c r="E319" t="inlineStr"/>
       <c r="F319" t="inlineStr">
         <is>
           <t>今</t>
@@ -10434,7 +10433,6 @@
           <t>はじめてきました</t>
         </is>
       </c>
-      <c r="H319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -10455,7 +10453,6 @@
           <t>いけちゃん</t>
         </is>
       </c>
-      <c r="E320" t="inlineStr"/>
       <c r="F320" t="inlineStr">
         <is>
           <t>すこーし</t>
@@ -10466,7 +10463,6 @@
           <t>きちゃ</t>
         </is>
       </c>
-      <c r="H320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -10487,7 +10483,6 @@
           <t>まや、とーり</t>
         </is>
       </c>
-      <c r="E321" t="inlineStr"/>
       <c r="F321" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -10498,7 +10493,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -10519,7 +10513,6 @@
           <t>たつ、かい</t>
         </is>
       </c>
-      <c r="E322" t="inlineStr"/>
       <c r="F322" t="inlineStr">
         <is>
           <t>いま</t>
@@ -10530,7 +10523,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="H322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -10551,7 +10543,6 @@
           <t>てくのちゃん</t>
         </is>
       </c>
-      <c r="E323" t="inlineStr"/>
       <c r="F323" t="inlineStr">
         <is>
           <t>おぺぺもって</t>
@@ -10562,7 +10553,6 @@
           <t>きたんご</t>
         </is>
       </c>
-      <c r="H323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -10583,7 +10573,6 @@
           <t>まいなちゅ</t>
         </is>
       </c>
-      <c r="E324" t="inlineStr"/>
       <c r="F324" t="inlineStr">
         <is>
           <t>今</t>
@@ -10594,7 +10583,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -10615,7 +10603,6 @@
           <t>あさみん、ことねえ</t>
         </is>
       </c>
-      <c r="E325" t="inlineStr"/>
       <c r="F325" t="inlineStr">
         <is>
           <t>今</t>
@@ -10626,7 +10613,6 @@
           <t>きまんた</t>
         </is>
       </c>
-      <c r="H325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -10647,7 +10633,6 @@
           <t>ぐっちゃん</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr"/>
       <c r="F326" t="inlineStr">
         <is>
           <t>おひさし</t>
@@ -10658,7 +10643,6 @@
           <t>きまんこ</t>
         </is>
       </c>
-      <c r="H326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -10679,7 +10663,6 @@
           <t>たろー、きょうちゃん</t>
         </is>
       </c>
-      <c r="E327" t="inlineStr"/>
       <c r="F327" t="inlineStr">
         <is>
           <t>初めて</t>
@@ -10690,7 +10673,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="H327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -10711,7 +10693,6 @@
           <t>りお、めい</t>
         </is>
       </c>
-      <c r="E328" t="inlineStr"/>
       <c r="F328" t="inlineStr">
         <is>
           <t>今</t>
@@ -10722,7 +10703,6 @@
           <t>きた！！！</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -10743,7 +10723,6 @@
           <t>まいまいまいまい</t>
         </is>
       </c>
-      <c r="E329" t="inlineStr"/>
       <c r="F329" t="inlineStr">
         <is>
           <t>しごおわ</t>
@@ -10754,7 +10733,6 @@
           <t>きました</t>
         </is>
       </c>
-      <c r="H329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -10775,7 +10753,6 @@
           <t>しん</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr"/>
       <c r="F330" t="inlineStr">
         <is>
           <t>モーニング</t>
@@ -10786,7 +10763,6 @@
           <t>おはようございます</t>
         </is>
       </c>
-      <c r="H330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -10859,7 +10835,6 @@
           <t>ゆう</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr"/>
       <c r="F332" t="inlineStr">
         <is>
           <t>初めてです</t>
@@ -10872,7 +10847,6 @@
 m(_ _)m</t>
         </is>
       </c>
-      <c r="H332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -10893,7 +10867,6 @@
           <t>ゆずき＆ましゅ</t>
         </is>
       </c>
-      <c r="E333" t="inlineStr"/>
       <c r="F333" t="inlineStr">
         <is>
           <t>2人で</t>
@@ -10904,7 +10877,6 @@
           <t>きたよ♪</t>
         </is>
       </c>
-      <c r="H333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -10925,7 +10897,6 @@
           <t>さと</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr"/>
       <c r="F334" t="inlineStr">
         <is>
           <t>今</t>
@@ -10936,7 +10907,6 @@
           <t>きたよ♪</t>
         </is>
       </c>
-      <c r="H334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -10957,7 +10927,6 @@
           <t>なお</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr"/>
       <c r="F335" t="inlineStr">
         <is>
           <t>しごおわで</t>
@@ -10968,7 +10937,6 @@
           <t>きた！</t>
         </is>
       </c>
-      <c r="H335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -10989,7 +10957,6 @@
           <t>こてっちゃん</t>
         </is>
       </c>
-      <c r="E336" t="inlineStr"/>
       <c r="F336" t="inlineStr">
         <is>
           <t>元気に</t>
@@ -11000,7 +10967,6 @@
           <t>キタタタタ</t>
         </is>
       </c>
-      <c r="H336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -11021,7 +10987,6 @@
           <t>さとるん</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr"/>
       <c r="F337" t="inlineStr">
         <is>
           <t>片付け</t>
@@ -11032,7 +10997,6 @@
           <t>終わったぜ</t>
         </is>
       </c>
-      <c r="H337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -11053,7 +11017,6 @@
           <t>かな</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr"/>
       <c r="F338" t="inlineStr">
         <is>
           <t>みんなおつかれ</t>
@@ -11064,7 +11027,6 @@
           <t>きたよー</t>
         </is>
       </c>
-      <c r="H338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -11085,7 +11047,6 @@
           <t>にゃんまげ</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr"/>
       <c r="F339" t="inlineStr">
         <is>
           <t>今きたで</t>
@@ -11096,7 +11057,6 @@
           <t>シャー</t>
         </is>
       </c>
-      <c r="H339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -11117,7 +11077,6 @@
           <t>おじき</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr"/>
       <c r="F340" t="inlineStr">
         <is>
           <t>朝まで</t>
@@ -11128,7 +11087,6 @@
           <t>ゴーゴー</t>
         </is>
       </c>
-      <c r="H340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -11149,7 +11107,6 @@
           <t>てくのちゃん</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr"/>
       <c r="F341" t="inlineStr">
         <is>
           <t>今</t>
@@ -11160,7 +11117,6 @@
           <t>きたわよん</t>
         </is>
       </c>
-      <c r="H341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -11181,7 +11137,6 @@
           <t>ふくちゃん、T山、まいまい</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr"/>
       <c r="F342" t="inlineStr">
         <is>
           <t>今</t>
@@ -11192,7 +11147,6 @@
           <t>来たぜっ</t>
         </is>
       </c>
-      <c r="H342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -11213,7 +11167,6 @@
           <t>なお</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr"/>
       <c r="F343" t="inlineStr">
         <is>
           <t>はじめて</t>
@@ -11224,7 +11177,6 @@
           <t>きました！</t>
         </is>
       </c>
-      <c r="H343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -11245,7 +11197,6 @@
           <t>zin、あんこ</t>
         </is>
       </c>
-      <c r="E344" t="inlineStr"/>
       <c r="F344" t="inlineStr">
         <is>
           <t>いま</t>
@@ -11256,7 +11207,6 @@
           <t>キッター</t>
         </is>
       </c>
-      <c r="H344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -11277,7 +11227,6 @@
           <t>まー</t>
         </is>
       </c>
-      <c r="E345" t="inlineStr"/>
       <c r="F345" t="inlineStr">
         <is>
           <t>忘れ物</t>
@@ -11288,7 +11237,6 @@
           <t>した人が、、、</t>
         </is>
       </c>
-      <c r="H345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -11342,6 +11290,250 @@
         </is>
       </c>
     </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>27396</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>18:48:40</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>彩</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr"/>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>オープンと同時に</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>行きますー、</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>27397</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>19:05:10</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr"/>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>早めに</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>来ましたー</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>27400</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>20:16:37</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>ケン、ツボ</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr"/>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>飲みおわ</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>きましたー</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>27402</v>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>21:05:01</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>ゆずきち</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>きたよー</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>27403</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>21:05:19</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>テクノっち</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>ワイちゃんも</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>きたよーん</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>27407</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>21:30:54</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>よちお</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr"/>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>今日は</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>ラッキーデイ♪</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>27409</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>03:40:06</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>★BAMBITCH★</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>欲求不満のポコチンハンター　える</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>★☆★朝までアゲアゲの火曜日営業が始まるわよ♪★☆★</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>本日9月1日の営業時間は♪
+オープン19:00！ラスト5:00なのよ☆
+担当は
+欲求不満のポコチンハンター　える
+なのよ♪
+どんな季節でも★BAMBITCH★は色気ムンムンで暑すぎる♪
+バンビッチでおもいっきりはじけちゃって（笑）
+精力は無くても性欲がある！？
+大人の憩いと禁断サークル盛りだくさん！
+憩いと交流の魔性の遊び場バンビッチは素敵な出会いを 提供いたします（笑)☆☆
+おつまみ等の持ち込みは自由なのでみんなで持ち寄ってお近づきのきっかけにどうぞ♪
+強制や無理強いは一切ございませんので楽しく遊びましょう♪
+宇都宮市宿郷1−12−9　カサブランカビル5F</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>img20260901034006.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11353,7 +11545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I418"/>
+  <dimension ref="A1:I425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29337,6 +29529,307 @@
       <c r="I418" t="inlineStr">
         <is>
           <t>した人が、、、</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>18:48:40</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>27396</v>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>彩</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>7</v>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>彩</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>オープンと同時に</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>行きますー、</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>19:05:10</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>27397</v>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>11</v>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>ひがん</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>早めに</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>来ましたー</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>20:16:37</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>27400</v>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>ケン</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>1</v>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>ケン、ツボ</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>飲みおわ</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>きましたー</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>20:16:37</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>27400</v>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>ツボ</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>1</v>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>ケン、ツボ</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>飲みおわ</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>きましたー</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>21:05:01</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>27402</v>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>ゆずきち</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>1</v>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>ゆずきち</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>遊びに</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>きたよー</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>21:05:19</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>27403</v>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>テクノっち</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>1</v>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>テクノっち</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>ワイちゃんも</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>きたよーん</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>21:30:54</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>27407</v>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>よちお</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>1</v>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>よちお</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>今日は</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>ラッキーデイ♪</t>
         </is>
       </c>
     </row>
@@ -29351,7 +29844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D268"/>
+  <dimension ref="A1:D273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29383,7 +29876,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -29392,7 +29885,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -29439,27 +29932,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>なお</t>
+          <t>彩</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ましゅ</t>
+          <t>なお</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -29467,19 +29960,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>テクノ</t>
+          <t>ましゅ</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -29487,19 +29980,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>彩</t>
+          <t>テクノ</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -29507,12 +30000,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -33439,7 +33932,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>ゆずき＆ましゅ</t>
+          <t>ゆずきち</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -33447,19 +33940,19 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>ゆぴ</t>
+          <t>ゆずき＆ましゅ</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -33467,19 +33960,19 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>ゆり</t>
+          <t>ゆぴ</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -33487,19 +33980,19 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>ゆん</t>
+          <t>ゆり</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -33507,19 +34000,19 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>らうら</t>
+          <t>ゆん</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -33539,7 +34032,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>らお</t>
+          <t>よちお</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -33547,19 +34040,19 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>りえ</t>
+          <t>らうら</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -33567,19 +34060,19 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>りく</t>
+          <t>らお</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -33587,19 +34080,19 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>りさ</t>
+          <t>りえ</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -33607,19 +34100,19 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>りゅう</t>
+          <t>りく</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -33627,19 +34120,19 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>りゅうくん</t>
+          <t>りさ</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -33647,19 +34140,19 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>りょうちゃん</t>
+          <t>りゅう</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -33667,19 +34160,19 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>りりこ</t>
+          <t>りゅうくん</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -33687,19 +34180,19 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>りん＆ゆち</t>
+          <t>りょうちゃん</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -33707,19 +34200,19 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>るい</t>
+          <t>りりこ</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -33727,19 +34220,19 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>れー</t>
+          <t>りん＆ゆち</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -33747,19 +34240,19 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ろくじ</t>
+          <t>るい</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -33767,19 +34260,19 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>アイちゃん</t>
+          <t>れー</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -33787,19 +34280,19 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>アキ</t>
+          <t>ろくじ</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -33807,19 +34300,19 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>アナルプリンス</t>
+          <t>アイちゃん</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -33827,19 +34320,19 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>オ・スー</t>
+          <t>アキ</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -33847,19 +34340,19 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>カミさん</t>
+          <t>アナルプリンス</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -33879,7 +34372,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>カモリ</t>
+          <t>オ・スー</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -33887,19 +34380,19 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>カー</t>
+          <t>カミさん</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -33907,19 +34400,19 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>キム</t>
+          <t>カモリ</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -33927,19 +34420,19 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>キムとどえむちゃん</t>
+          <t>カー</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -33947,19 +34440,19 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>キムとドMまゆ</t>
+          <t>キム</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -33967,19 +34460,19 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>キムと奴隷</t>
+          <t>キムとどえむちゃん</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -33987,19 +34480,19 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>キムと新しい奴隷ちゃん</t>
+          <t>キムとドMまゆ</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -34007,19 +34500,19 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>コオリ</t>
+          <t>キムと奴隷</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -34027,19 +34520,19 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>ザッキー</t>
+          <t>キムと新しい奴隷ちゃん</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -34047,19 +34540,19 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>シュンヤ</t>
+          <t>ケン</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -34067,19 +34560,19 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>ジャッキー</t>
+          <t>コオリ</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -34087,19 +34580,19 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>ジョーカー</t>
+          <t>ザッキー</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -34107,19 +34600,19 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>タカ</t>
+          <t>シュンヤ</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -34127,19 +34620,19 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>タカス</t>
+          <t>ジャッキー</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -34147,19 +34640,19 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>ダイキ</t>
+          <t>ジョーカー</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -34167,19 +34660,19 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>ダイゴ</t>
+          <t>タカ</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -34187,19 +34680,19 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>ダイチ</t>
+          <t>タカス</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -34207,19 +34700,19 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>テクノとポチ</t>
+          <t>ダイキ</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -34227,19 +34720,19 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>トニー・トニー・チョッパー</t>
+          <t>ダイゴ</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -34247,19 +34740,19 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>ナカヤマヤ</t>
+          <t>ダイチ</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -34267,19 +34760,19 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>ニト</t>
+          <t>ツボ</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -34287,19 +34780,19 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>フジ</t>
+          <t>テクノっち</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -34307,19 +34800,19 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>ボンタ</t>
+          <t>テクノとポチ</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -34327,19 +34820,19 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>マイナス</t>
+          <t>トニー・トニー・チョッパー</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -34347,19 +34840,19 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>マサ</t>
+          <t>ナカヤマヤ</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -34367,19 +34860,19 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>マッチョ</t>
+          <t>ニト</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -34387,19 +34880,19 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>マナティ</t>
+          <t>フジ</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -34419,7 +34912,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>ミッシ</t>
+          <t>ボンタ</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -34427,19 +34920,19 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>モジャ</t>
+          <t>マイナス</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -34447,19 +34940,19 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>ユキ</t>
+          <t>マサ</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -34467,19 +34960,19 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>ユッキー</t>
+          <t>マッチョ</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -34487,19 +34980,19 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>ヨシヤ</t>
+          <t>マナティ</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -34507,19 +35000,19 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>リョウ</t>
+          <t>ミッシ</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -34539,7 +35032,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>ロタポジ</t>
+          <t>モジャ</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -34547,19 +35040,19 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>僕と私</t>
+          <t>ユキ</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -34567,19 +35060,19 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>名無し</t>
+          <t>ユッキー</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -34587,19 +35080,19 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>大塚</t>
+          <t>ヨシヤ</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -34607,19 +35100,19 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>女子三人衆</t>
+          <t>リョウ</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -34627,19 +35120,19 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>海砂利水魚</t>
+          <t>ロタポジ</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -34647,19 +35140,19 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>絶</t>
+          <t>僕と私</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -34667,19 +35160,19 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>赤ちゃん</t>
+          <t>名無し</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -34687,30 +35180,130 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
+          <t>大塚</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>1</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>女子三人衆</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>1</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>海砂利水魚</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>1</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>絶</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>1</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>赤ちゃん</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>1</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
           <t>高田</t>
         </is>
       </c>
-      <c r="B268" t="n">
-        <v>1</v>
-      </c>
-      <c r="C268" t="inlineStr">
+      <c r="B273" t="n">
+        <v>1</v>
+      </c>
+      <c r="C273" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="D268" t="inlineStr">
+      <c r="D273" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -34754,10 +35347,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C2" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -35110,10 +35703,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C20" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
@@ -35123,10 +35716,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C21" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22">
@@ -35136,10 +35729,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C22" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23">
@@ -35149,10 +35742,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C23" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24">
@@ -35224,13 +35817,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="C2" t="n">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="D2" t="n">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -35244,7 +35837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36812,12 +37405,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>タカ</t>
+          <t>ケン</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>タク</t>
+          <t>ツボ</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -36827,12 +37420,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>タカス</t>
+          <t>タカ</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>マサ</t>
+          <t>タク</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -36842,12 +37435,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>タク</t>
+          <t>タカス</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>リョウ</t>
+          <t>マサ</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -36857,12 +37450,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ダイキ</t>
+          <t>タク</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ミッシ</t>
+          <t>リョウ</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -36872,15 +37465,30 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
+          <t>ダイキ</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>ミッシ</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
           <t>テクノ</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>ミコト</t>
         </is>
       </c>
-      <c r="C109" t="n">
+      <c r="C110" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>